<commit_message>
Presupuestos completos, reportes de compras y presupuestos, portal de clientes
</commit_message>
<xml_diff>
--- a/public/ejemplos/lista-distribuidora-norte.xlsx
+++ b/public/ejemplos/lista-distribuidora-norte.xlsx
@@ -621,7 +621,7 @@
         <v>8</v>
       </c>
       <c r="D5">
-        <v>44.94</v>
+        <v>44.12</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -635,7 +635,7 @@
         <v>8</v>
       </c>
       <c r="D6">
-        <v>9.96</v>
+        <v>9.68</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -663,7 +663,7 @@
         <v>8</v>
       </c>
       <c r="D8">
-        <v>21.15</v>
+        <v>20.54</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -677,7 +677,7 @@
         <v>19</v>
       </c>
       <c r="D9">
-        <v>105.83</v>
+        <v>104.98</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -691,7 +691,7 @@
         <v>19</v>
       </c>
       <c r="D10">
-        <v>226.38</v>
+        <v>232.88999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -719,7 +719,7 @@
         <v>19</v>
       </c>
       <c r="D12">
-        <v>3733.19999999999982</v>
+        <v>3614.19999999999982</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -747,7 +747,7 @@
         <v>30</v>
       </c>
       <c r="D14">
-        <v>10760.39999999999964</v>
+        <v>10348.79999999999927</v>
       </c>
       <c r="E14">
         <v>4.0</v>
@@ -764,7 +764,7 @@
         <v>30</v>
       </c>
       <c r="D15">
-        <v>15834.0</v>
+        <v>16109.5</v>
       </c>
       <c r="E15">
         <v>4.0</v>
@@ -781,7 +781,7 @@
         <v>30</v>
       </c>
       <c r="D16">
-        <v>409.25999999999999</v>
+        <v>419.51999999999998</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -795,7 +795,7 @@
         <v>30</v>
       </c>
       <c r="D17">
-        <v>480.24000000000001</v>
+        <v>478.86000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -823,7 +823,7 @@
         <v>30</v>
       </c>
       <c r="D19">
-        <v>22743.0</v>
+        <v>21987.0</v>
       </c>
       <c r="E19">
         <v>4.0</v>
@@ -840,7 +840,7 @@
         <v>19</v>
       </c>
       <c r="D20">
-        <v>495.44999999999999</v>
+        <v>496.35000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -854,7 +854,7 @@
         <v>19</v>
       </c>
       <c r="D21">
-        <v>3301.5</v>
+        <v>3329.40000000000009</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -882,7 +882,7 @@
         <v>47</v>
       </c>
       <c r="D23">
-        <v>5595.19999999999982</v>
+        <v>5543.19999999999982</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -896,7 +896,7 @@
         <v>19</v>
       </c>
       <c r="D24">
-        <v>9879.0</v>
+        <v>9736.60000000000036</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -924,7 +924,7 @@
         <v>19</v>
       </c>
       <c r="D26">
-        <v>4293.89999999999964</v>
+        <v>4141.80000000000018</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -938,7 +938,7 @@
         <v>19</v>
       </c>
       <c r="D27">
-        <v>35168.0</v>
+        <v>35104.0</v>
       </c>
       <c r="E27">
         <v>25.0</v>
@@ -955,7 +955,7 @@
         <v>19</v>
       </c>
       <c r="D28">
-        <v>4864.5</v>
+        <v>4842.0</v>
       </c>
     </row>
     <row r="29" spans="1:5">

</xml_diff>